<commit_message>
docs(bom): set spreadsheet author to Aaradhya Dev Tamrakar
</commit_message>
<xml_diff>
--- a/docs/SPARK_Component_Order_Form.xlsx
+++ b/docs/SPARK_Component_Order_Form.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="17985" windowHeight="7748" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
@@ -23,55 +23,20 @@
     <numFmt numFmtId="168" formatCode="0&quot; lot&quot;"/>
     <numFmt numFmtId="169" formatCode="0&quot; lot for 2 nodes&quot;"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <name val="&quot;Times New Roman&quot;"/>
-      <charset val="1"/>
-      <b val="1"/>
-      <color rgb="FF000000"/>
-      <sz val="14"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <name val="Arial"/>
       <charset val="1"/>
       <family val="2"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <charset val="1"/>
-      <family val="2"/>
-      <b val="1"/>
       <color theme="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="&quot;Times New Roman&quot;"/>
-      <charset val="1"/>
-      <b val="1"/>
-      <color rgb="FF000000"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <charset val="1"/>
-      <family val="2"/>
-      <b val="1"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <charset val="1"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color rgb="FF000000"/>
       <sz val="10"/>
     </font>
     <font>
@@ -84,6 +49,47 @@
     <font>
       <name val="&quot;Times New Roman&quot;"/>
       <charset val="1"/>
+      <family val="2"/>
+      <color rgb="FF000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="&quot;Times New Roman&quot;"/>
+      <charset val="1"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FF000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="&quot;Times New Roman&quot;"/>
+      <charset val="1"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FF000000"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="1"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <charset val="1"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <charset val="1"/>
+      <family val="2"/>
+      <b val="1"/>
       <color rgb="FF000000"/>
       <sz val="10"/>
     </font>
@@ -96,11 +102,8 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <b val="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="1"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -109,7 +112,9 @@
       <patternFill/>
     </fill>
     <fill>
-      <patternFill patternType="gray125"/>
+      <patternFill patternType="gray125">
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -128,16 +133,29 @@
     </border>
     <border>
       <left style="thin">
-        <color auto="1"/>
+        <color indexed="64"/>
       </left>
       <right style="thin">
-        <color auto="1"/>
+        <color indexed="64"/>
       </right>
       <top style="thin">
-        <color auto="1"/>
+        <color indexed="64"/>
       </top>
       <bottom style="thin">
-        <color auto="1"/>
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
@@ -145,7 +163,7 @@
       <left/>
       <right/>
       <top style="thin">
-        <color auto="1"/>
+        <color indexed="64"/>
       </top>
       <bottom/>
       <diagonal/>
@@ -153,22 +171,22 @@
     <border>
       <left/>
       <right style="thin">
-        <color auto="1"/>
+        <color indexed="64"/>
       </right>
       <top style="thin">
-        <color auto="1"/>
+        <color indexed="64"/>
       </top>
       <bottom/>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color auto="1"/>
+        <color indexed="64"/>
       </left>
       <right/>
       <top/>
       <bottom style="thin">
-        <color auto="1"/>
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
@@ -177,18 +195,18 @@
       <right/>
       <top/>
       <bottom style="thin">
-        <color auto="1"/>
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left/>
       <right style="thin">
-        <color auto="1"/>
+        <color indexed="64"/>
       </right>
       <top/>
       <bottom style="thin">
-        <color auto="1"/>
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
@@ -196,29 +214,16 @@
       <left/>
       <right/>
       <top style="thin">
-        <color auto="1"/>
+        <color indexed="64"/>
       </top>
       <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color auto="1"/>
+        <color indexed="64"/>
       </left>
       <right/>
       <top/>
@@ -228,7 +233,7 @@
     <border>
       <left/>
       <right style="thin">
-        <color auto="1"/>
+        <color indexed="64"/>
       </right>
       <top/>
       <bottom/>
@@ -238,36 +243,36 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -282,56 +287,50 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -340,32 +339,32 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -475,7 +474,7 @@
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office Theme">
       <a:dk1>
         <a:srgbClr val="000000"/>
       </a:dk1>
@@ -513,84 +512,48 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office Theme">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Calibri Light"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme>
+    <a:fmtScheme name="Craft">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:tint val="67000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:tint val="73000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:tint val="81000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect/>
-        </a:gradFill>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:shade val="78000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect/>
-        </a:gradFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
         <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
@@ -609,35 +572,11 @@
           <a:schemeClr val="phClr"/>
         </a:solidFill>
         <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-          </a:schemeClr>
+          <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect/>
-        </a:gradFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
@@ -653,23 +592,22 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N27"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9.06640625" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9.00390625" defaultRowHeight="14.25" customHeight="1"/>
   <cols>
-    <col width="5.06640625" customWidth="1" style="1" min="1" max="1"/>
-    <col width="43.06640625" customWidth="1" style="1" min="2" max="2"/>
-    <col width="8.1328125" customWidth="1" style="1" min="3" max="3"/>
-    <col width="11.53125" customWidth="1" style="1" min="4" max="4"/>
-    <col width="13.06640625" customWidth="1" style="1" min="5" max="5"/>
-    <col width="8.73046875" customWidth="1" style="1" min="6" max="6"/>
-    <col width="33.73046875" customWidth="1" style="1" min="7" max="7"/>
-    <col width="8.1328125" customWidth="1" style="1" min="8" max="8"/>
-    <col width="8.9296875" customWidth="1" style="1" min="9" max="9"/>
-    <col width="8.796875" customWidth="1" style="1" min="10" max="10"/>
-    <col width="9.06640625" customWidth="1" style="1" min="11" max="11"/>
-    <col width="25.73046875" customWidth="1" style="1" min="12" max="12"/>
-    <col width="14.86328125" customWidth="1" style="1" min="13" max="13"/>
-    <col width="9.06640625" customWidth="1" style="1" min="14" max="14"/>
-    <col width="9.06640625" customWidth="1" style="1" min="15" max="16384"/>
+    <col width="5.00390625" customWidth="1" style="1" min="1" max="1"/>
+    <col width="43.00390625" customWidth="1" style="1" min="2" max="2"/>
+    <col width="8.140625" customWidth="1" style="1" min="3" max="3"/>
+    <col width="11.57421875" customWidth="1" style="1" min="4" max="4"/>
+    <col width="13.00390625" customWidth="1" style="1" min="5" max="5"/>
+    <col width="8.7109375" customWidth="1" style="1" min="6" max="6"/>
+    <col width="33.7109375" customWidth="1" style="1" min="7" max="7"/>
+    <col width="8.140625" customWidth="1" style="1" min="8" max="8"/>
+    <col width="9.00390625" customWidth="1" style="1" min="9" max="9"/>
+    <col width="8.8515625" customWidth="1" style="1" min="10" max="10"/>
+    <col width="9.00390625" customWidth="1" style="1" min="11" max="11"/>
+    <col width="25.7109375" customWidth="1" style="1" min="12" max="12"/>
+    <col width="14.8515625" customWidth="1" style="1" min="13" max="13"/>
+    <col width="9.00390625" customWidth="1" style="1" min="14" max="16384"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -678,30 +616,30 @@
           <t>Project name: SPARK — Wearable Fall Detection System</t>
         </is>
       </c>
-      <c r="B1" s="35" t="n"/>
-      <c r="C1" s="35" t="n"/>
-      <c r="D1" s="35" t="n"/>
-      <c r="E1" s="35" t="n"/>
-      <c r="F1" s="35" t="n"/>
-      <c r="G1" s="35" t="n"/>
-      <c r="H1" s="35" t="n"/>
-      <c r="I1" s="35" t="n"/>
-      <c r="J1" s="36" t="n"/>
+      <c r="B1" s="33" t="n"/>
+      <c r="C1" s="33" t="n"/>
+      <c r="D1" s="33" t="n"/>
+      <c r="E1" s="33" t="n"/>
+      <c r="F1" s="33" t="n"/>
+      <c r="G1" s="33" t="n"/>
+      <c r="H1" s="33" t="n"/>
+      <c r="I1" s="33" t="n"/>
+      <c r="J1" s="34" t="n"/>
       <c r="K1" s="2" t="n"/>
       <c r="L1" s="2" t="n"/>
       <c r="M1" s="2" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="37" t="n"/>
-      <c r="B2" s="38" t="n"/>
-      <c r="C2" s="38" t="n"/>
-      <c r="D2" s="38" t="n"/>
-      <c r="E2" s="38" t="n"/>
-      <c r="F2" s="38" t="n"/>
-      <c r="G2" s="38" t="n"/>
-      <c r="H2" s="38" t="n"/>
-      <c r="I2" s="38" t="n"/>
-      <c r="J2" s="39" t="n"/>
+      <c r="A2" s="35" t="n"/>
+      <c r="B2" s="36" t="n"/>
+      <c r="C2" s="36" t="n"/>
+      <c r="D2" s="36" t="n"/>
+      <c r="E2" s="36" t="n"/>
+      <c r="F2" s="36" t="n"/>
+      <c r="G2" s="36" t="n"/>
+      <c r="H2" s="36" t="n"/>
+      <c r="I2" s="36" t="n"/>
+      <c r="J2" s="37" t="n"/>
       <c r="K2" s="2" t="n"/>
       <c r="L2" s="2" t="n"/>
       <c r="M2" s="2" t="n"/>
@@ -713,17 +651,17 @@
           <t>Components List</t>
         </is>
       </c>
-      <c r="C3" s="40" t="n"/>
-      <c r="D3" s="40" t="n"/>
-      <c r="E3" s="40" t="n"/>
+      <c r="C3" s="38" t="n"/>
+      <c r="D3" s="38" t="n"/>
+      <c r="E3" s="38" t="n"/>
       <c r="F3" s="15" t="n"/>
       <c r="G3" s="19" t="n"/>
-      <c r="H3" s="21" t="inlineStr">
+      <c r="H3" s="20" t="inlineStr">
         <is>
           <t>TO ORDER</t>
         </is>
       </c>
-      <c r="I3" s="40" t="n"/>
+      <c r="I3" s="38" t="n"/>
       <c r="J3" s="15" t="n"/>
       <c r="K3" s="2" t="n"/>
       <c r="L3" s="2" t="n"/>
@@ -735,47 +673,47 @@
           <t>S.N.</t>
         </is>
       </c>
-      <c r="B4" s="21" t="inlineStr">
+      <c r="B4" s="20" t="inlineStr">
         <is>
           <t>Components with main features</t>
         </is>
       </c>
-      <c r="C4" s="21" t="inlineStr">
+      <c r="C4" s="20" t="inlineStr">
         <is>
           <t>Quantity</t>
         </is>
       </c>
-      <c r="D4" s="21" t="inlineStr">
+      <c r="D4" s="20" t="inlineStr">
         <is>
           <t>ISSUED (NRs.)</t>
         </is>
       </c>
-      <c r="E4" s="21" t="inlineStr">
+      <c r="E4" s="20" t="inlineStr">
         <is>
           <t>Unit Cost (NRs.)</t>
         </is>
       </c>
-      <c r="F4" s="21" t="inlineStr">
+      <c r="F4" s="20" t="inlineStr">
         <is>
           <t>Total Cost</t>
         </is>
       </c>
-      <c r="G4" s="21" t="inlineStr">
+      <c r="G4" s="20" t="inlineStr">
         <is>
           <t>Availability</t>
         </is>
       </c>
-      <c r="H4" s="21" t="inlineStr">
+      <c r="H4" s="20" t="inlineStr">
         <is>
           <t>Quantity</t>
         </is>
       </c>
-      <c r="I4" s="21" t="inlineStr">
+      <c r="I4" s="20" t="inlineStr">
         <is>
           <t>Unit Cost (NRs.)</t>
         </is>
       </c>
-      <c r="J4" s="21" t="inlineStr">
+      <c r="J4" s="20" t="inlineStr">
         <is>
           <t>Total Cost (NRs.)</t>
         </is>
@@ -784,7 +722,7 @@
       <c r="L4" s="2" t="n"/>
       <c r="M4" s="2" t="n"/>
     </row>
-    <row r="5">
+    <row r="5" ht="40.5" customHeight="1">
       <c r="A5" s="12" t="n">
         <v>1</v>
       </c>
@@ -830,7 +768,7 @@
       <c r="M5" s="15" t="n"/>
       <c r="N5" s="6" t="n"/>
     </row>
-    <row r="6">
+    <row r="6" ht="15" customHeight="1">
       <c r="A6" s="12" t="n">
         <v>2</v>
       </c>
@@ -878,7 +816,7 @@
       </c>
       <c r="N6" s="9" t="n"/>
     </row>
-    <row r="7">
+    <row r="7" ht="28.5" customHeight="1">
       <c r="A7" s="12" t="n">
         <v>3</v>
       </c>
@@ -926,7 +864,7 @@
       </c>
       <c r="N7" s="9" t="n"/>
     </row>
-    <row r="8">
+    <row r="8" ht="28.5" customHeight="1">
       <c r="A8" s="12" t="n">
         <v>4</v>
       </c>
@@ -974,7 +912,7 @@
       </c>
       <c r="N8" s="9" t="n"/>
     </row>
-    <row r="9">
+    <row r="9" ht="15" customHeight="1">
       <c r="A9" s="12" t="n">
         <v>5</v>
       </c>
@@ -1022,7 +960,7 @@
       </c>
       <c r="N9" s="9" t="n"/>
     </row>
-    <row r="10">
+    <row r="10" ht="28.5" customHeight="1">
       <c r="A10" s="12" t="n">
         <v>6</v>
       </c>
@@ -1069,7 +1007,7 @@
         <v>9841576746</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" ht="28.5" customHeight="1">
       <c r="A11" s="12" t="n">
         <v>7</v>
       </c>
@@ -1096,7 +1034,7 @@
           <t>KEC Makerspace / vendor TBD</t>
         </is>
       </c>
-      <c r="H11" s="41" t="n">
+      <c r="H11" s="39" t="n">
         <v>1</v>
       </c>
       <c r="I11" s="3" t="n">
@@ -1111,7 +1049,7 @@
       <c r="M11" s="10" t="n"/>
       <c r="N11" s="9" t="n"/>
     </row>
-    <row r="12">
+    <row r="12" ht="53.25" customHeight="1">
       <c r="A12" s="12" t="n">
         <v>8</v>
       </c>
@@ -1152,7 +1090,7 @@
       <c r="L12" s="11" t="n"/>
       <c r="M12" s="2" t="n"/>
     </row>
-    <row r="13">
+    <row r="13" ht="40.5" customHeight="1">
       <c r="A13" s="12" t="n">
         <v>9</v>
       </c>
@@ -1179,7 +1117,7 @@
           <t>Himalayan Solutions</t>
         </is>
       </c>
-      <c r="H13" s="42" t="n">
+      <c r="H13" s="40" t="n">
         <v>2</v>
       </c>
       <c r="I13" s="3" t="n">
@@ -1193,7 +1131,7 @@
       <c r="L13" s="11" t="n"/>
       <c r="M13" s="11" t="n"/>
     </row>
-    <row r="14">
+    <row r="14" ht="40.5" customHeight="1">
       <c r="A14" s="12" t="n">
         <v>10</v>
       </c>
@@ -1220,7 +1158,7 @@
           <t>Himalayan Solutions</t>
         </is>
       </c>
-      <c r="H14" s="43" t="n">
+      <c r="H14" s="41" t="n">
         <v>1</v>
       </c>
       <c r="I14" s="3" t="n">
@@ -1262,7 +1200,7 @@
           <t>Daraz Nepal</t>
         </is>
       </c>
-      <c r="H15" s="44" t="n">
+      <c r="H15" s="42" t="n">
         <v>20</v>
       </c>
       <c r="I15" s="3" t="n">
@@ -1273,7 +1211,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" customFormat="1" s="34">
+    <row r="16" ht="28.5" customFormat="1" customHeight="1" s="32">
       <c r="A16" s="12" t="n">
         <v>12</v>
       </c>
@@ -1311,7 +1249,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" ht="14.25" customHeight="1">
+    <row r="17" ht="33" customHeight="1">
       <c r="A17" s="12" t="n">
         <v>13</v>
       </c>
@@ -1338,7 +1276,7 @@
           <t>Himalayan Solutions / Daraz</t>
         </is>
       </c>
-      <c r="H17" s="45" t="n">
+      <c r="H17" s="43" t="n">
         <v>1</v>
       </c>
       <c r="I17" s="3" t="n">
@@ -1349,7 +1287,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" ht="14.25" customHeight="1">
+    <row r="18" ht="62.25" customHeight="1">
       <c r="A18" s="12" t="n">
         <v>14</v>
       </c>
@@ -1376,7 +1314,7 @@
           <t>Himalayan Solutions</t>
         </is>
       </c>
-      <c r="H18" s="46" t="n">
+      <c r="H18" s="44" t="n">
         <v>1</v>
       </c>
       <c r="I18" s="3" t="n">
@@ -1386,11 +1324,11 @@
         <f>H18*I18</f>
         <v/>
       </c>
-      <c r="K18" s="33" t="n"/>
-      <c r="L18" s="33" t="n"/>
-      <c r="M18" s="33" t="n"/>
-    </row>
-    <row r="19" ht="14.25" customHeight="1">
+      <c r="K18" s="31" t="n"/>
+      <c r="L18" s="31" t="n"/>
+      <c r="M18" s="31" t="n"/>
+    </row>
+    <row r="19" ht="33" customHeight="1">
       <c r="A19" s="12" t="n">
         <v>15</v>
       </c>
@@ -1417,7 +1355,7 @@
           <t>Applicable suppliers</t>
         </is>
       </c>
-      <c r="H19" s="45" t="n">
+      <c r="H19" s="43" t="n">
         <v>1</v>
       </c>
       <c r="I19" s="3" t="n">
@@ -1431,28 +1369,28 @@
       <c r="L19" s="11" t="n"/>
       <c r="M19" s="11" t="n"/>
     </row>
-    <row r="20">
-      <c r="A20" s="31" t="n"/>
-      <c r="B20" s="30" t="n"/>
-      <c r="C20" s="31" t="n"/>
-      <c r="D20" s="31" t="inlineStr">
+    <row r="20" ht="15" customHeight="1">
+      <c r="A20" s="28" t="n"/>
+      <c r="B20" s="29" t="n"/>
+      <c r="C20" s="28" t="n"/>
+      <c r="D20" s="28" t="inlineStr">
         <is>
           <t>Priced subtotal</t>
         </is>
       </c>
       <c r="E20" s="15" t="n"/>
-      <c r="F20" s="31">
+      <c r="F20" s="28">
         <f>SUM(F5:F19)</f>
         <v/>
       </c>
-      <c r="G20" s="31" t="n"/>
-      <c r="H20" s="31" t="inlineStr">
+      <c r="G20" s="28" t="n"/>
+      <c r="H20" s="28" t="inlineStr">
         <is>
           <t>Priced subtotal</t>
         </is>
       </c>
       <c r="I20" s="15" t="n"/>
-      <c r="J20" s="31">
+      <c r="J20" s="28">
         <f>SUM(J5:J19)</f>
         <v/>
       </c>
@@ -1460,28 +1398,28 @@
       <c r="L20" s="11" t="n"/>
       <c r="M20" s="11" t="n"/>
     </row>
-    <row r="21">
-      <c r="A21" s="31" t="n"/>
-      <c r="B21" s="30" t="n"/>
-      <c r="C21" s="31" t="n"/>
-      <c r="D21" s="31" t="inlineStr">
+    <row r="21" ht="15" customHeight="1">
+      <c r="A21" s="28" t="n"/>
+      <c r="B21" s="29" t="n"/>
+      <c r="C21" s="28" t="n"/>
+      <c r="D21" s="28" t="inlineStr">
         <is>
           <t>Grand total</t>
         </is>
       </c>
       <c r="E21" s="15" t="n"/>
-      <c r="F21" s="31">
+      <c r="F21" s="28">
         <f>F20</f>
         <v/>
       </c>
-      <c r="G21" s="31" t="n"/>
-      <c r="H21" s="31" t="inlineStr">
+      <c r="G21" s="28" t="n"/>
+      <c r="H21" s="28" t="inlineStr">
         <is>
           <t>Grand total</t>
         </is>
       </c>
       <c r="I21" s="15" t="n"/>
-      <c r="J21" s="31">
+      <c r="J21" s="28">
         <f>J20</f>
         <v/>
       </c>
@@ -1498,35 +1436,35 @@
       <c r="M22" s="11" t="n"/>
     </row>
     <row r="23">
-      <c r="B23" s="47" t="inlineStr">
+      <c r="B23" s="45" t="inlineStr">
         <is>
           <t>Notes for submission:</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="48" t="inlineStr">
+      <c r="B24" s="46" t="inlineStr">
         <is>
           <t>- Row 1 includes three 50 cm USB-C data+power cables, so the separate cable purchase is removed.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="B25" s="48" t="inlineStr">
+      <c r="B25" s="46" t="inlineStr">
         <is>
           <t>- Qty 3 across ESP32-S3, MPU6050, TP4056, 5V boost converter, and SPDT switch ensures 2 active nodes (1 Wrist + 1 Waist reference) + 1 complete spare chain.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="48" t="inlineStr">
+      <c r="B26" s="46" t="inlineStr">
         <is>
           <t>- Row 9 (M-F/F-F jumpers) + Row 14 (2.54 mm female headers, solder/flux, foam/Kapton tape, waist belt) eliminate Day-1 bring-up &amp; assembly blockers.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="B27" s="48" t="inlineStr">
+      <c r="B27" s="46" t="inlineStr">
         <is>
           <t>- All 15 BOM lines are fully costed: Grand Total NPR 17,677 (or NPR 14,037 with per-gram KEC Makerspace TPU printing).</t>
         </is>
@@ -1543,8 +1481,8 @@
     <mergeCell ref="H3:J3"/>
     <mergeCell ref="D21:E21"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
+  <pageMargins left="0.699999988079071" right="0.699999988079071" top="0.75" bottom="0.75" header="0.5118110179901123" footer="0.5118110179901123"/>
+  <pageSetup orientation="portrait" paperSize="9"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>